<commit_message>
Audit 10 more reports against filings (123 figures): Alphabet net cash corrected (SpaceX stake was counted twice; value $249 to $245, still Hold); clarifications for Alphabet, Meta and RTX; audit log now 185 figures in 15 reports
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR3LbNEqqh1NJpsKSu2JUT
</commit_message>
<xml_diff>
--- a/data/models/alphabet.xlsx
+++ b/data/models/alphabet.xlsx
@@ -1080,15 +1080,15 @@
       </c>
       <c r="B21" s="21" t="n">
         <f aca="false">Bear!$B$43</f>
-        <v>139.059569487102</v>
+        <v>134.994263364653</v>
       </c>
       <c r="C21" s="21" t="n">
         <f aca="false">Base!$B$43</f>
-        <v>249.12108551844</v>
+        <v>245.055779395991</v>
       </c>
       <c r="D21" s="21" t="n">
         <f aca="false">Bull!$B$43</f>
-        <v>379.791258521498</v>
+        <v>375.725952399049</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="C23" s="22" t="n">
         <f aca="false">SUMPRODUCT(B21:D21,B22:D22)</f>
-        <v>254.27324976137</v>
+        <v>250.207943638921</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="C25" s="23" t="n">
         <f aca="false">C23/C24-1</f>
-        <v>-0.215738542466936</v>
+        <v>-0.228277269635059</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C29" s="26" t="n">
         <f aca="false">(SUMPRODUCT(Base!$B$32:$K$32,1/(1+B29)^(Base!$B$24:$K$24-0.5))+Base!$K$29*(1+Base!$B$10)*(1-Base!$B$14)*(1-Base!$B$10/Base!$B$16)/(B29-Base!$B$10)/(1+B29)^9.5+Base!$B$19)/Base!$B$20</f>
-        <v>323.802706739709</v>
+        <v>319.73740061726</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="C30" s="26" t="n">
         <f aca="false">(SUMPRODUCT(Base!$B$32:$K$32,1/(1+B30)^(Base!$B$24:$K$24-0.5))+Base!$K$29*(1+Base!$B$10)*(1-Base!$B$14)*(1-Base!$B$10/Base!$B$16)/(B30-Base!$B$10)/(1+B30)^9.5+Base!$B$19)/Base!$B$20</f>
-        <v>296.482775880237</v>
+        <v>292.417469757788</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="C31" s="26" t="n">
         <f aca="false">(SUMPRODUCT(Base!$B$32:$K$32,1/(1+B31)^(Base!$B$24:$K$24-0.5))+Base!$K$29*(1+Base!$B$10)*(1-Base!$B$14)*(1-Base!$B$10/Base!$B$16)/(B31-Base!$B$10)/(1+B31)^9.5+Base!$B$19)/Base!$B$20</f>
-        <v>273.404944990774</v>
+        <v>269.339638868325</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="C32" s="26" t="n">
         <f aca="false">(SUMPRODUCT(Base!$B$32:$K$32,1/(1+B32)^(Base!$B$24:$K$24-0.5))+Base!$K$29*(1+Base!$B$10)*(1-Base!$B$14)*(1-Base!$B$10/Base!$B$16)/(B32-Base!$B$10)/(1+B32)^9.5+Base!$B$19)/Base!$B$20</f>
-        <v>253.659561789285</v>
+        <v>249.594255666836</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="C33" s="26" t="n">
         <f aca="false">(SUMPRODUCT(Base!$B$32:$K$32,1/(1+B33)^(Base!$B$24:$K$24-0.5))+Base!$K$29*(1+Base!$B$10)*(1-Base!$B$14)*(1-Base!$B$10/Base!$B$16)/(B33-Base!$B$10)/(1+B33)^9.5+Base!$B$19)/Base!$B$20</f>
-        <v>236.579550303484</v>
+        <v>232.514244181035</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1449,7 +1449,7 @@
         <v>58</v>
       </c>
       <c r="B19" s="15" t="n">
-        <v>318.4</v>
+        <v>268.6</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>17</v>
@@ -2047,7 +2047,7 @@
       </c>
       <c r="B42" s="14" t="n">
         <f aca="false">B41+$B$19</f>
-        <v>3051.73329760089</v>
+        <v>3001.93329760089</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2056,7 +2056,7 @@
       </c>
       <c r="B43" s="22" t="n">
         <f aca="false">B42/$B$20</f>
-        <v>249.12108551844</v>
+        <v>245.055779395991</v>
       </c>
     </row>
   </sheetData>
@@ -2278,7 +2278,7 @@
         <v>58</v>
       </c>
       <c r="B19" s="15" t="n">
-        <v>318.4</v>
+        <v>268.6</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>17</v>
@@ -2876,7 +2876,7 @@
       </c>
       <c r="B42" s="14" t="n">
         <f aca="false">B41+$B$19</f>
-        <v>1703.479726217</v>
+        <v>1653.679726217</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2885,7 +2885,7 @@
       </c>
       <c r="B43" s="22" t="n">
         <f aca="false">B42/$B$20</f>
-        <v>139.059569487102</v>
+        <v>134.994263364653</v>
       </c>
     </row>
   </sheetData>
@@ -3107,7 +3107,7 @@
         <v>58</v>
       </c>
       <c r="B19" s="15" t="n">
-        <v>318.4</v>
+        <v>268.6</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>17</v>
@@ -3705,7 +3705,7 @@
       </c>
       <c r="B42" s="14" t="n">
         <f aca="false">B41+$B$19</f>
-        <v>4652.44291688835</v>
+        <v>4602.64291688835</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="B43" s="22" t="n">
         <f aca="false">B42/$B$20</f>
-        <v>379.791258521498</v>
+        <v>375.725952399049</v>
       </c>
     </row>
   </sheetData>

</xml_diff>